<commit_message>
Rework STTM Excel: use lowest-level schema.table source references, add Mapping Type and Notes columns
</commit_message>
<xml_diff>
--- a/STTM_location_d.xlsx
+++ b/STTM_location_d.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="212">
   <si>
     <t>Attribute</t>
   </si>
@@ -57,73 +57,67 @@
     <t>Data Filter</t>
   </si>
   <si>
-    <t>TO_TIMESTAMP('{{data_filter_end_dttm}}', 'yyyymmdd HH24:MI:SS') &gt;= erp_start_date</t>
-  </si>
-  <si>
-    <t>Source Alias</t>
-  </si>
-  <si>
-    <t>Source Table</t>
+    <t>TO_TIMESTAMP('{{data_filter_end_dttm}}', 'yyyymmdd HH24:MI:SS') &gt;= erp_start_date (from XYZdata.Oracle_Erp_start_Date)</t>
   </si>
   <si>
     <t>Schema</t>
   </si>
   <si>
+    <t>Table</t>
+  </si>
+  <si>
+    <t>SQL Alias</t>
+  </si>
+  <si>
     <t>Description</t>
   </si>
   <si>
-    <t>location_code_list</t>
-  </si>
-  <si>
-    <t>InventoryOrgParametersPVO + ffmcenter</t>
-  </si>
-  <si>
-    <t>oracle_erp / order_management_service</t>
-  </si>
-  <si>
-    <t>UNION of ERP org codes and OMS fulfillment center names; provides the master list of location codes</t>
+    <t>oracle_erp</t>
   </si>
   <si>
     <t>InventoryOrgParametersPVO</t>
   </si>
   <si>
-    <t>oracle_erp</t>
-  </si>
-  <si>
-    <t>Oracle ERP inventory org parameters (org code, enabled flag, business unit)</t>
+    <t>InventoryOrgParametersPVO / location_code_list (UNION branch 1)</t>
+  </si>
+  <si>
+    <t>Oracle ERP inventory org parameters — provides org code (location_code), enabled flag, business unit, legal entity name</t>
+  </si>
+  <si>
+    <t>order_management_service</t>
+  </si>
+  <si>
+    <t>ffmcenter</t>
+  </si>
+  <si>
+    <t>ffmcenter / location_code_list (UNION branch 2)</t>
+  </si>
+  <si>
+    <t>OMS fulfillment center master — provides id, name (used as location_code), type, address, SLA days, pick settings</t>
   </si>
   <si>
     <t>INV_ORG_PARAMETERS</t>
   </si>
   <si>
-    <t>Oracle ERP inventory org attributes (warehouse type, EZ Ship flag)</t>
+    <t>Oracle ERP inventory org attributes — provides warehouse type (ATTRIBUTE1) and EZ Ship flag</t>
   </si>
   <si>
     <t>hr_locations</t>
   </si>
   <si>
-    <t>Oracle HR location master (address, city, state, postal code)</t>
-  </si>
-  <si>
-    <t>ffmcenter</t>
-  </si>
-  <si>
-    <t>order_management_service</t>
-  </si>
-  <si>
-    <t>OMS fulfillment center master (id, name, type, address, SLA days)</t>
+    <t>Oracle HR location master — provides address, city, state/region, postal code</t>
+  </si>
+  <si>
+    <t>denver_retirement</t>
+  </si>
+  <si>
+    <t>ffmcenter_raw</t>
   </si>
   <si>
     <t>ffmcenter_hist</t>
   </si>
   <si>
-    <t>ffmcenter_raw</t>
-  </si>
-  <si>
-    <t>denver_retirement</t>
-  </si>
-  <si>
-    <t>Historical fulfillment center data</t>
+    <t>Historical fulfillment center data (joined but not currently used in SELECT output)</t>
   </si>
   <si>
     <t>fcs</t>
@@ -132,19 +126,37 @@
     <t>fulfillment_center</t>
   </si>
   <si>
-    <t>FCS fulfillment center details (enabled flag, display name, address, SLA)</t>
-  </si>
-  <si>
-    <t>tmp_location_id</t>
-  </si>
-  <si>
-    <t>location_d + codecombinationpvo</t>
-  </si>
-  <si>
-    <t>dw / oracle_erp</t>
-  </si>
-  <si>
-    <t>Temporary table resolving oracle_location_id per location_code</t>
+    <t>FCS fulfillment center details — provides enabled flag, display name, address, SLA days, type</t>
+  </si>
+  <si>
+    <t>location_d</t>
+  </si>
+  <si>
+    <t>tmp_location_id (branch 1) / ps (UPDATE/INSERT)</t>
+  </si>
+  <si>
+    <t>Target dimension table — used to resolve existing oracle_location_id and as the UPDATE/INSERT target</t>
+  </si>
+  <si>
+    <t>codecombinationpvo</t>
+  </si>
+  <si>
+    <t>erp (in tmp_location_id branch 2)</t>
+  </si>
+  <si>
+    <t>ERP code combination — used to parse oracle_location_id from codecombinationdescription via regex</t>
+  </si>
+  <si>
+    <t>XYZdata</t>
+  </si>
+  <si>
+    <t>Oracle_Erp_start_Date</t>
+  </si>
+  <si>
+    <t>(subquery in WHERE clause)</t>
+  </si>
+  <si>
+    <t>Provides erp_start_date used in the data filter condition</t>
   </si>
   <si>
     <t>#</t>
@@ -156,7 +168,7 @@
     <t>Target Data Type</t>
   </si>
   <si>
-    <t>Source Table(s)</t>
+    <t>Source Schema.Table</t>
   </si>
   <si>
     <t>Source Column(s)</t>
@@ -180,49 +192,57 @@
     <t>VARCHAR</t>
   </si>
   <si>
-    <t>Direct — derived from UNION of OrgOrganizationDefinitionsPOrganizationCode (ERP) and ffmcenter.name (OMS)</t>
+    <t xml:space="preserve">oracle_erp.InventoryOrgParametersPVO
+order_management_service.ffmcenter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OrgOrganizationDefinitionsPOrganizationCode (ERP branch)
+name (OMS branch)</t>
+  </si>
+  <si>
+    <t>UNION of DISTINCT OrgOrganizationDefinitionsPOrganizationCode from oracle_erp.InventoryOrgParametersPVO and DISTINCT name from order_management_service.ffmcenter. The combined result forms the master list of location codes.</t>
+  </si>
+  <si>
+    <t>Derived/Computed</t>
+  </si>
+  <si>
+    <t>NOT NULL</t>
+  </si>
+  <si>
+    <t>Natural/business key; grain of the dimension. Derived from a UNION subquery aliased as location_code_list.</t>
+  </si>
+  <si>
+    <t>location_key</t>
+  </si>
+  <si>
+    <t>INTEGER</t>
+  </si>
+  <si>
+    <t>ROW_NUMBER() OVER (ORDER BY 'location_key') + (SELECT MAX(location_key) FROM dw.location_d). Applied only on INSERT of new rows.</t>
+  </si>
+  <si>
+    <t>Surrogate key generated only on INSERT; offset from current MAX to avoid collisions with existing keys.</t>
+  </si>
+  <si>
+    <t>fulfillment_center_id</t>
+  </si>
+  <si>
+    <t>order_management_service.ffmcenter</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>Direct — ffmcenter.id. Aggregated with MAX() in UPDATE/INSERT SELECT.</t>
   </si>
   <si>
     <t>Direct Mapping</t>
   </si>
   <si>
-    <t>NOT NULL</t>
-  </si>
-  <si>
-    <t>Natural/business key; grain of the dimension table</t>
-  </si>
-  <si>
-    <t>location_key</t>
-  </si>
-  <si>
-    <t>INTEGER</t>
-  </si>
-  <si>
-    <t>Surrogate key: ROW_NUMBER() OVER (ORDER BY 'location_key') + MAX(location_key) from existing dw.location_d. Applied only on INSERT of new rows.</t>
-  </si>
-  <si>
-    <t>Derived/Computed</t>
-  </si>
-  <si>
-    <t>Surrogate key generated only on INSERT; offset from current MAX to avoid collisions</t>
-  </si>
-  <si>
-    <t>fulfillment_center_id</t>
-  </si>
-  <si>
-    <t>order_management_service.ffmcenter</t>
-  </si>
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>Direct — ffmcenter.id. Aggregated with MAX() in final SELECT.</t>
-  </si>
-  <si>
     <t>NULLABLE</t>
   </si>
   <si>
-    <t>MAX() aggregation used to collapse multiple rows per location_code</t>
+    <t>MAX() aggregation used to collapse multiple staging rows per location_code.</t>
   </si>
   <si>
     <t>fulfillment_active</t>
@@ -246,19 +266,24 @@
     <t>location_display_name</t>
   </si>
   <si>
-    <t>fcs.fulfillment_center, oracle_erp.hr_locations, InventoryOrgParametersPVO</t>
-  </si>
-  <si>
-    <t>display_name, LegalEntityPEOName, region_2, InvOrgNamePEOName</t>
-  </si>
-  <si>
-    <t>NVL(LegalEntityPEOName || ' (' || hr_locations.region_2 || ' - ' || InvOrgNamePEOName || ')', fcs.display_name) — prefers ERP-derived name; falls back to FCS display name. Aggregated with MAX().</t>
+    <t xml:space="preserve">oracle_erp.InventoryOrgParametersPVO
+oracle_erp.hr_locations
+fcs.fulfillment_center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LegalEntityPEOName (InventoryOrgParametersPVO)
+InvOrgNamePEOName (InventoryOrgParametersPVO)
+region_2 (hr_locations)
+display_name (fcs.fulfillment_center)</t>
+  </si>
+  <si>
+    <t>NVL(LegalEntityPEOName || ' (' || hr_locations.region_2 || ' - ' || InvOrgNamePEOName || ')', fcs.display_name). ERP-derived composite name preferred; falls back to fcs.display_name when ERP name is NULL. Aggregated with MAX().</t>
   </si>
   <si>
     <t>Conditional Logic/ CASE Statement</t>
   </si>
   <si>
-    <t>ERP-derived name preferred; NVL fallback to fcs.display_name</t>
+    <t>NVL acts as conditional: ERP composite name takes priority; fcs.display_name is the fallback.</t>
   </si>
   <si>
     <t>location_active_warehouse</t>
@@ -276,7 +301,7 @@
     <t>CASE WHEN OrgOrganizationDefinitionsPInventoryEnabledFlag = 'Y' THEN 1 ELSE 0 END. Aggregated with MAX().</t>
   </si>
   <si>
-    <t>Flag encoded as integer: 1 = active, 0 = inactive</t>
+    <t>Flag encoded as integer: 1 = active ('Y'), 0 = inactive (any other value).</t>
   </si>
   <si>
     <t>location_warehouse_type</t>
@@ -291,40 +316,44 @@
     <t>CASE WHEN ATTRIBUTE1 IN ('Retail','Pharmacy') THEN 0 WHEN ATTRIBUTE1 = 'Freezer' THEN 1 WHEN ATTRIBUTE1 = 'Cross Dock' THEN 3 END. Aggregated with MAX().</t>
   </si>
   <si>
-    <t>Retail/Pharmacy=0, Freezer=1, Cross Dock=3; NULL for unrecognised values</t>
+    <t>Retail/Pharmacy=0, Freezer=1, Cross Dock=3. NULL for unrecognised ATTRIBUTE1 values. Joined via INV_ORG_PARAMETERS.ORGANIZATION_ID = InventoryOrgParametersPVO.OrganizationId.</t>
   </si>
   <si>
     <t>location_address1</t>
   </si>
   <si>
-    <t>fcs.fulfillment_center, oracle_erp.hr_locations</t>
-  </si>
-  <si>
-    <t>address_line1, address_line_1</t>
-  </si>
-  <si>
-    <t>CASE WHEN TYPE = 'DROPSHIP' THEN fcs.address_line1 ELSE hr_locations.address_line_1 END. DROPSHIP locations use FCS address; all others use HR address. Aggregated with MAX().</t>
-  </si>
-  <si>
-    <t>Address source priority: DROPSHIP → FCS; all others → Oracle HR</t>
+    <t xml:space="preserve">fcs.fulfillment_center
+oracle_erp.hr_locations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">address_line1 (fcs.fulfillment_center)
+address_line_1 (oracle_erp.hr_locations)</t>
+  </si>
+  <si>
+    <t>CASE WHEN TYPE = 'DROPSHIP' THEN fcs.address_line1 ELSE hr_locations.address_line_1 END. Aggregated with MAX().</t>
+  </si>
+  <si>
+    <t>TYPE comes from order_management_service.ffmcenter. DROPSHIP → FCS address; all other types → Oracle HR address.</t>
   </si>
   <si>
     <t>location_city</t>
   </si>
   <si>
-    <t>city, town_or_city</t>
+    <t xml:space="preserve">city (fcs.fulfillment_center)
+town_or_city (oracle_erp.hr_locations)</t>
   </si>
   <si>
     <t>CASE WHEN TYPE = 'DROPSHIP' THEN fcs.city ELSE hr_locations.town_or_city END. Aggregated with MAX().</t>
   </si>
   <si>
-    <t>Same address source priority rule as location_address1</t>
+    <t>Same address source priority rule as location_address1.</t>
   </si>
   <si>
     <t>location_post_code</t>
   </si>
   <si>
-    <t>postal_code</t>
+    <t xml:space="preserve">postal_code (fcs.fulfillment_center)
+postal_code (oracle_erp.hr_locations)</t>
   </si>
   <si>
     <t>CASE WHEN TYPE = 'DROPSHIP' THEN fcs.postal_code ELSE hr_locations.postal_code END. Aggregated with MAX().</t>
@@ -345,7 +374,7 @@
     <t>maxnumpick</t>
   </si>
   <si>
-    <t>Direct — maxnumpick. Aggregated with MAX().</t>
+    <t>Direct — ffmcenter.maxnumpick. Aggregated with MAX().</t>
   </si>
   <si>
     <t>fulfillment_center_pick_delay</t>
@@ -354,7 +383,7 @@
     <t>pick_delay</t>
   </si>
   <si>
-    <t>Direct — pick_delay. Aggregated with MAX().</t>
+    <t>Direct — ffmcenter.pick_delay. Aggregated with MAX().</t>
   </si>
   <si>
     <t>fulfillment_center_storage_rate</t>
@@ -366,13 +395,13 @@
     <t>(none)</t>
   </si>
   <si>
-    <t>Hardcoded NULL — not currently sourced. Aggregated with MAX().</t>
+    <t>NULL — hardcoded literal NULL. Aggregated with MAX().</t>
   </si>
   <si>
     <t>Hardcoded/Null</t>
   </si>
   <si>
-    <t>Placeholder column; no source data available at this time</t>
+    <t>Placeholder column; no source data available at this time.</t>
   </si>
   <si>
     <t>fulfillment_center_default_shipping_offset</t>
@@ -381,52 +410,69 @@
     <t>default_ship_offset</t>
   </si>
   <si>
-    <t>Direct — default_ship_offset. Aggregated with MAX().</t>
+    <t>Direct — ffmcenter.default_ship_offset. Aggregated with MAX().</t>
   </si>
   <si>
     <t>fulfillment_center_mark_for_delete</t>
   </si>
   <si>
-    <t>NOT fcs.fc_enabled — inverted active flag. Aggregated with MAX().</t>
-  </si>
-  <si>
-    <t>Logical inverse of fulfillment_active; derived from the same source column fc_enabled</t>
+    <t>NOT fcs.fc_enabled — logical NOT of the active flag. Aggregated with MAX().</t>
+  </si>
+  <si>
+    <t>Logical inverse of fulfillment_active; both columns derive from the same source column fcs.fc_enabled.</t>
   </si>
   <si>
     <t>legal_company_description</t>
   </si>
   <si>
-    <t>location_code, dw_site_id</t>
-  </si>
-  <si>
-    <t>CASE on location_code / dw_site_id: 'SDF1'→'Petsmart', 'SDF3'→'Wholesale', 'STK1'→'XYZ Virtual Care', 'STK2'→'Stark Services PLLC', dw_site_id=60→'Retail Canada', else 'Retail'. Aggregated with MAX().</t>
-  </si>
-  <si>
-    <t>Specific overrides for known location codes; Canada site (dw_site_id=60) maps to Retail Canada</t>
+    <t xml:space="preserve">OrgOrganizationDefinitionsPOrganizationCode (location_code)
+businessunitpeoname → dw_site_id (derived in UNION subquery)</t>
+  </si>
+  <si>
+    <t>CASE WHEN location_code = 'SDF1' THEN 'Petsmart' WHEN location_code = 'SDF3' THEN 'Wholesale' WHEN location_code = 'STK1' THEN 'XYZ Virtual Care' WHEN location_code = 'STK2' THEN 'Stark Services PLLC' WHEN dw_site_id = 60 THEN 'Retail Canada' ELSE 'Retail' END. Aggregated with MAX().</t>
+  </si>
+  <si>
+    <t>dw_site_id is derived in the UNION subquery: businessunitpeoname = 'XYZ CA BU' → 60, else 10. Specific location_code overrides take priority over site-level rule.</t>
   </si>
   <si>
     <t>product_company_description</t>
   </si>
   <si>
-    <t>location_code_list, fcs.fulfillment_center</t>
-  </si>
-  <si>
-    <t>location_code, dw_site_id, type</t>
-  </si>
-  <si>
-    <t>CASE: STK%→'XYZ Healthcare Services', PHARMA+site 10→'XYZ Pharmacy', PHARMA+site 60→'XYZ Pharmacy Canada', site 60→'XYZ Canada', else 'XYZ'. Aggregated with MAX().</t>
-  </si>
-  <si>
-    <t>Multi-condition CASE using location_code pattern, dw_site_id, and fulfillment center type</t>
+    <t xml:space="preserve">oracle_erp.InventoryOrgParametersPVO
+order_management_service.ffmcenter
+fcs.fulfillment_center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OrgOrganizationDefinitionsPOrganizationCode (location_code)
+businessunitpeoname → dw_site_id (derived)
+type (fcs.fulfillment_center)</t>
+  </si>
+  <si>
+    <t>CASE WHEN location_code LIKE 'STK%' THEN 'XYZ Healthcare Services' WHEN fcs.type = 'PHARMA' AND dw_site_id = 10 THEN 'XYZ Pharmacy' WHEN fcs.type = 'PHARMA' AND dw_site_id = 60 THEN 'XYZ Pharmacy Canada' WHEN dw_site_id = 60 THEN 'XYZ Canada' ELSE 'XYZ' END. Aggregated with MAX().</t>
+  </si>
+  <si>
+    <t>Multi-condition CASE using location_code pattern match, dw_site_id (derived from businessunitpeoname), and fcs.type.</t>
   </si>
   <si>
     <t>oracle_location_id</t>
   </si>
   <si>
-    <t>Resolved via temp table tmp_location_id (see Temp Table sheet). Joined on location_code. Aggregated with MAX().</t>
-  </si>
-  <si>
-    <t>See "Temp Table" sheet for full resolution logic using UNION of existing DW values and ERP code combination parsing</t>
+    <t xml:space="preserve">dw.location_d
+oracle_erp.codecombinationpvo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">oracle_location_id (dw.location_d — branch 1)
+codecombinationsegment3 (oracle_erp.codecombinationpvo — branch 2)
+codecombinationdescription (oracle_erp.codecombinationpvo — branch 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resolved via temp table tmp_location_id (UNION of two branches):
+Branch 1: SELECT DISTINCT oracle_location_id, location_code FROM dw.location_d WHERE oracle_location_id IS NOT NULL AND oracle_location_id NOT IN (codecombinationpvo derived IDs).
+Branch 2: SELECT DISTINCT codecombinationsegment3::int, split_part(regexp_substr(codecombinationdescription, '-[a-zA-Z] \d-'), '-', 2) FROM oracle_erp.codecombinationpvo JOIN dw.location_d.
+Joined to staging on location_code. Aggregated with MAX().</t>
+  </si>
+  <si>
+    <t>See "Temp Table" sheet for full resolution logic. Branch 2 parses location_code from codecombinationdescription using regex -[a-zA-Z] \d- and splits on -.</t>
   </si>
   <si>
     <t>location_ez_ship_flag</t>
@@ -435,10 +481,14 @@
     <t>CASE WHEN ATTRIBUTE1 = 'EZ Ship' THEN TRUE ELSE FALSE END. Aggregated with MAX().</t>
   </si>
   <si>
+    <t>Joined via INV_ORG_PARAMETERS.ORGANIZATION_ID = InventoryOrgParametersPVO.OrganizationId.</t>
+  </si>
+  <si>
     <t>location_address2</t>
   </si>
   <si>
-    <t>address_line2, address_line_2</t>
+    <t xml:space="preserve">address_line2 (fcs.fulfillment_center)
+address_line_2 (oracle_erp.hr_locations)</t>
   </si>
   <si>
     <t>CASE WHEN TYPE = 'DROPSHIP' THEN fcs.address_line2 ELSE hr_locations.address_line_2 END. Aggregated with MAX().</t>
@@ -450,13 +500,14 @@
     <t>VARCHAR(2)</t>
   </si>
   <si>
-    <t>state, region_2</t>
-  </si>
-  <si>
-    <t>UPPER(LEFT(CASE WHEN TYPE = 'DROPSHIP' THEN fcs.state ELSE hr_locations.region_2 END, 2)) — upper-cased 2-character state code. Aggregated with MAX().</t>
-  </si>
-  <si>
-    <t>Always upper-cased and truncated to 2 characters regardless of source value length</t>
+    <t xml:space="preserve">state (fcs.fulfillment_center)
+region_2 (oracle_erp.hr_locations)</t>
+  </si>
+  <si>
+    <t>UPPER(LEFT(CASE WHEN TYPE = 'DROPSHIP' THEN fcs.state ELSE hr_locations.region_2 END, 2)). Aggregated with MAX().</t>
+  </si>
+  <si>
+    <t>Always upper-cased and truncated to 2 characters. Same DROPSHIP/non-DROPSHIP address priority as other address columns.</t>
   </si>
   <si>
     <t>location_ship_sla_days</t>
@@ -471,7 +522,10 @@
     <t>Branch</t>
   </si>
   <si>
-    <t>Source</t>
+    <t>Source Tables</t>
+  </si>
+  <si>
+    <t>Source Columns</t>
   </si>
   <si>
     <t>Logic</t>
@@ -480,16 +534,24 @@
     <t>Branch 1</t>
   </si>
   <si>
-    <t>Select oracle_location_id and location_code where oracle_location_id IS NOT NULL AND the ID does not already exist in the ERP codecombinationpvo join result (avoids duplicates).</t>
+    <t>oracle_location_id, location_code</t>
+  </si>
+  <si>
+    <t>SELECT DISTINCT oracle_location_id::int, location_code FROM dw.location_d WHERE oracle_location_id IS NOT NULL AND oracle_location_id NOT IN (SELECT DISTINCT codecombinationsegment3::int FROM oracle_erp.codecombinationpvo JOIN dw.location_d ON split_part(regexp_substr(codecombinationdescription, '-[a-zA-Z] \d-'), '-', 2) = location_code). Preserves existing DW values that are not superseded by ERP parsing.</t>
   </si>
   <si>
     <t>Branch 2</t>
   </si>
   <si>
-    <t>oracle_erp.codecombinationpvo JOIN dw.location_d</t>
-  </si>
-  <si>
-    <t>Extract codecombinationsegment3::int as oracle_location_id; extract location_code by parsing codecombinationdescription with regex -[a-zA-Z] \d- and splitting on -.</t>
+    <t xml:space="preserve">oracle_erp.codecombinationpvo
+dw.location_d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">codecombinationsegment3 → oracle_location_id
+codecombinationdescription → location_code (via regex)</t>
+  </si>
+  <si>
+    <t>SELECT DISTINCT codecombinationsegment3::int AS oracle_location_id, split_part(regexp_substr(codecombinationdescription, '-[a-zA-Z] \d-'), '-', 2) AS location_code FROM oracle_erp.codecombinationpvo erp JOIN dw.location_d loc ON split_part(regexp_substr(erp.codecombinationdescription, '-[a-zA-Z] \d-'), '-', 2) = loc.location_code. Extracts oracle_location_id from ERP code combinations by parsing the description field.</t>
   </si>
   <si>
     <t>Step</t>
@@ -504,7 +566,7 @@
     <t>Populate Staging (staging.location_ds)</t>
   </si>
   <si>
-    <t>Truncate/replace staging table with the full SELECT from source systems. Data filter: only process if {{data_filter_end_dttm}} &gt;= ERP start date.</t>
+    <t>INSERT INTO staging.location_ds: full SELECT from source systems (oracle_erp.InventoryOrgParametersPVO, order_management_service.ffmcenter, oracle_erp.INV_ORG_PARAMETERS, oracle_erp.hr_locations, denver_retirement.ffmcenter_raw, fcs.fulfillment_center). Data filter: only process if TO_TIMESTAMP('{{data_filter_end_dttm}}', 'yyyymmdd HH24:MI:SS') &gt;= erp_start_date from XYZdata.Oracle_Erp_start_Date.</t>
   </si>
   <si>
     <t>Step 2</t>
@@ -513,7 +575,7 @@
     <t>Build tmp_location_id</t>
   </si>
   <si>
-    <t>Resolve oracle_location_id per location_code using UNION of existing DW values and ERP code combination parsing.</t>
+    <t>Create local temporary table tmp_location_id (ON COMMIT PRESERVE ROWS). UNION of: (1) existing oracle_location_id values from dw.location_d not superseded by ERP parsing, and (2) oracle_location_id values parsed from oracle_erp.codecombinationpvo via regex on codecombinationdescription.</t>
   </si>
   <si>
     <t>Step 3</t>
@@ -522,7 +584,7 @@
     <t>UPDATE existing rows in dw.location_d</t>
   </si>
   <si>
-    <t>Match on location_code. All non-key attributes are overwritten with the latest values from staging (aggregated via MAX()).</t>
+    <t>UPDATE dw.location_d SET all non-key columns from a subquery on staging.location_ds LEFT JOIN tmp_location_id, grouped by location_code with MAX() aggregation. Match condition: ps.location_code = ls.location_code.</t>
   </si>
   <si>
     <t>Step 4</t>
@@ -531,7 +593,7 @@
     <t>INSERT new rows into dw.location_d</t>
   </si>
   <si>
-    <t>Only rows where location_code does NOT already exist in dw.location_d (LEFT JOIN + WHERE ps.location_code IS NULL). location_key is generated as a sequential surrogate key offset from the current maximum.</t>
+    <t>INSERT INTO dw.location_d: rows from staging.location_ds LEFT JOIN tmp_location_id (grouped, MAX() aggregated) LEFT JOIN dw.location_d WHERE ps.location_code IS NULL (i.e. location_code does not yet exist in target). location_key generated as ROW_NUMBER() OVER (ORDER BY 'location_key') + MAX(location_key) from dw.location_d.</t>
   </si>
   <si>
     <t>Step 5</t>
@@ -540,7 +602,7 @@
     <t>COMMIT</t>
   </si>
   <si>
-    <t>Commit the transaction.</t>
+    <t>COMMIT the transaction to persist all changes.</t>
   </si>
   <si>
     <t>Rule</t>
@@ -549,61 +611,73 @@
     <t>Address source priority</t>
   </si>
   <si>
-    <t>DROPSHIP type → use FCS address fields; all other types → use Oracle HR address fields</t>
+    <t>DROPSHIP type (from order_management_service.ffmcenter.type) → use fcs.fulfillment_center address fields; all other types → use oracle_erp.hr_locations address fields</t>
   </si>
   <si>
     <t>Display name priority</t>
   </si>
   <si>
-    <t>ERP-derived name (LegalEntityPEOName + region_2 + InvOrgNamePEOName) preferred; falls back to fcs.display_name via NVL</t>
+    <t>ERP-derived composite name (LegalEntityPEOName || ' (' || hr_locations.region_2 || ' - ' || InvOrgNamePEOName || ')') preferred; falls back to fcs.display_name via NVL when ERP name is NULL</t>
   </si>
   <si>
     <t>Warehouse type encoding</t>
   </si>
   <si>
-    <t>Retail/Pharmacy = 0, Freezer = 1, Cross Dock = 3</t>
+    <t>oracle_erp.INV_ORG_PARAMETERS.ATTRIBUTE1: Retail/Pharmacy = 0, Freezer = 1, Cross Dock = 3; NULL for unrecognised values</t>
   </si>
   <si>
     <t>Active warehouse flag</t>
   </si>
   <si>
-    <t>1 if OrgOrganizationDefinitionsPInventoryEnabledFlag = 'Y', else 0</t>
+    <t>oracle_erp.InventoryOrgParametersPVO.OrgOrganizationDefinitionsPInventoryEnabledFlag: 1 if 'Y', else 0</t>
   </si>
   <si>
     <t>Mark for delete</t>
   </si>
   <si>
-    <t>Inverse of fcs.fc_enabled</t>
+    <t>Logical NOT of fcs.fulfillment_center.fc_enabled</t>
   </si>
   <si>
     <t>Legal company</t>
   </si>
   <si>
-    <t>Specific overrides for SDF1, SDF3, STK1, STK2; Canada site (60) = 'Retail Canada'; default = 'Retail'</t>
+    <t>Specific overrides for SDF1→Petsmart, SDF3→Wholesale, STK1→XYZ Virtual Care, STK2→Stark Services PLLC; dw_site_id=60 (XYZ CA BU) → 'Retail Canada'; default → 'Retail'</t>
   </si>
   <si>
     <t>Product company</t>
   </si>
   <si>
-    <t>STK% codes → 'XYZ Healthcare Services'; PHARMA type by site; Canada site → 'XYZ Canada'; default → 'XYZ'</t>
+    <t>STK% location codes → 'XYZ Healthcare Services'; fcs.type='PHARMA' + site 10 → 'XYZ Pharmacy'; fcs.type='PHARMA' + site 60 → 'XYZ Pharmacy Canada'; site 60 → 'XYZ Canada'; default → 'XYZ'</t>
   </si>
   <si>
     <t>State code</t>
   </si>
   <si>
-    <t>Always upper-cased and truncated to 2 characters</t>
+    <t>Always UPPER-cased and truncated to 2 characters via UPPER(LEFT(..., 2))</t>
   </si>
   <si>
     <t>Storage rate</t>
   </si>
   <si>
-    <t>Always NULL (not yet sourced)</t>
+    <t>Always NULL — hardcoded literal; no source data available</t>
   </si>
   <si>
     <t>Surrogate key</t>
   </si>
   <si>
-    <t>Generated only on INSERT; offset from current MAX to avoid collisions</t>
+    <t>Generated only on INSERT; ROW_NUMBER() OVER (ORDER BY 'location_key') + MAX(location_key) from dw.location_d to avoid collisions</t>
+  </si>
+  <si>
+    <t>dw_site_id derivation</t>
+  </si>
+  <si>
+    <t>Derived inside the UNION subquery: businessunitpeoname = 'XYZ CA BU' → 60, else 10. Used in legal_company_description and product_company_description CASE logic.</t>
+  </si>
+  <si>
+    <t>Data filter</t>
+  </si>
+  <si>
+    <t>Only process records where TO_TIMESTAMP('{{data_filter_end_dttm}}', 'yyyymmdd HH24:MI:SS') &gt;= erp_start_date from XYZdata.Oracle_Erp_start_Date</t>
   </si>
 </sst>
 </file>
@@ -638,12 +712,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor rgb="FFBDD7EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFBDD7EE"/>
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -676,7 +750,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -684,10 +758,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1031,7 +1116,7 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
-    <col min="2" max="2" width="70" customWidth="1"/>
+    <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -1098,12 +1183,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="2" width="45" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="70" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1128,10 +1213,10 @@
       <c r="B2" t="s">
         <v>19</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1140,97 +1225,111 @@
         <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" t="s">
         <v>23</v>
       </c>
-      <c r="D3" t="s">
+      <c r="C3" s="2" t="s">
         <v>24</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" t="s">
         <v>26</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" t="s">
         <v>28</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" t="s">
         <v>31</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D7" t="s">
-        <v>35</v>
+      <c r="D7" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="B8" t="s">
         <v>37</v>
       </c>
-      <c r="C8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="C8" s="2" t="s">
         <v>38</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
         <v>40</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="2" t="s">
         <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1247,707 +1346,708 @@
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="5" width="45" customWidth="1"/>
-    <col min="6" max="6" width="80" customWidth="1"/>
-    <col min="7" max="7" width="30" customWidth="1"/>
+    <col min="4" max="4" width="50" customWidth="1"/>
+    <col min="5" max="5" width="45" customWidth="1"/>
+    <col min="6" max="6" width="85" customWidth="1"/>
+    <col min="7" max="7" width="32" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="60" customWidth="1"/>
+    <col min="9" max="9" width="65" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>52</v>
+      <c r="B2" s="3" t="s">
+        <v>56</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>18</v>
+        <v>58</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="H2" t="s">
-        <v>56</v>
+        <v>60</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>58</v>
+      <c r="B3" s="3" t="s">
+        <v>64</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="H3" t="s">
-        <v>56</v>
+      <c r="H3" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>63</v>
+      <c r="B4" s="3" t="s">
+        <v>68</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="H4" t="s">
-        <v>67</v>
+        <v>71</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
-        <v>69</v>
+      <c r="B5" s="3" t="s">
+        <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="H5" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="H5" t="s">
-        <v>67</v>
-      </c>
       <c r="I5" s="2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
-        <v>75</v>
+      <c r="B6" s="3" t="s">
+        <v>81</v>
       </c>
       <c r="C6" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="H6" t="s">
-        <v>67</v>
+        <v>84</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
-        <v>81</v>
+      <c r="B7" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="C7" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="G7" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="G7" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="H7" t="s">
-        <v>67</v>
+      <c r="H7" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
-        <v>87</v>
+      <c r="B8" s="3" t="s">
+        <v>93</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="H8" t="s">
-        <v>67</v>
+        <v>96</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
-        <v>92</v>
+      <c r="B9" s="3" t="s">
+        <v>98</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="H9" t="s">
-        <v>67</v>
+        <v>101</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
-        <v>97</v>
+      <c r="B10" s="3" t="s">
+        <v>103</v>
       </c>
       <c r="C10" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="H10" t="s">
-        <v>67</v>
+        <v>105</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
-        <v>101</v>
+      <c r="B11" s="3" t="s">
+        <v>107</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="H11" t="s">
-        <v>67</v>
+        <v>109</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
-        <v>104</v>
+      <c r="B12" s="3" t="s">
+        <v>110</v>
       </c>
       <c r="C12" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="H12" t="s">
-        <v>67</v>
+        <v>112</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" t="s">
-        <v>107</v>
+      <c r="B13" s="3" t="s">
+        <v>113</v>
       </c>
       <c r="C13" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="H13" t="s">
-        <v>67</v>
+        <v>115</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" t="s">
-        <v>110</v>
+      <c r="B14" s="3" t="s">
+        <v>116</v>
       </c>
       <c r="C14" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="H14" t="s">
-        <v>67</v>
+        <v>118</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15" t="s">
-        <v>113</v>
+      <c r="B15" s="3" t="s">
+        <v>119</v>
       </c>
       <c r="C15" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="H15" t="s">
-        <v>67</v>
+        <v>122</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16" t="s">
-        <v>119</v>
+      <c r="B16" s="3" t="s">
+        <v>125</v>
       </c>
       <c r="C16" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="H16" t="s">
-        <v>67</v>
+        <v>127</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
-      <c r="B17" t="s">
-        <v>122</v>
+      <c r="B17" s="3" t="s">
+        <v>128</v>
       </c>
       <c r="C17" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="G17" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="H17" t="s">
-        <v>67</v>
+      <c r="H17" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
-      <c r="B18" t="s">
-        <v>125</v>
+      <c r="B18" s="3" t="s">
+        <v>131</v>
       </c>
       <c r="C18" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>18</v>
+        <v>58</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="H18" t="s">
-        <v>67</v>
+        <v>133</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
-      <c r="B19" t="s">
-        <v>129</v>
+      <c r="B19" s="3" t="s">
+        <v>135</v>
       </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="H19" t="s">
-        <v>67</v>
+        <v>138</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
-      <c r="B20" t="s">
-        <v>134</v>
+      <c r="B20" s="3" t="s">
+        <v>140</v>
       </c>
       <c r="C20" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>39</v>
+        <v>141</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G20" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="H20" t="s">
-        <v>67</v>
+      <c r="H20" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21" t="s">
-        <v>137</v>
+      <c r="B21" s="3" t="s">
+        <v>145</v>
       </c>
       <c r="C21" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="H21" t="s">
-        <v>67</v>
+        <v>146</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>74</v>
+        <v>147</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22" t="s">
-        <v>139</v>
+      <c r="B22" s="3" t="s">
+        <v>148</v>
       </c>
       <c r="C22" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="H22" t="s">
-        <v>67</v>
+        <v>150</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23" t="s">
-        <v>142</v>
+      <c r="B23" s="3" t="s">
+        <v>151</v>
       </c>
       <c r="C23" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="G23" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="H23" t="s">
-        <v>67</v>
+      <c r="H23" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
-      <c r="B24" t="s">
-        <v>147</v>
+      <c r="B24" s="3" t="s">
+        <v>156</v>
       </c>
       <c r="C24" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="H24" t="s">
-        <v>67</v>
+        <v>158</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1958,45 +2058,54 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="35" customWidth="1"/>
-    <col min="3" max="3" width="90" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="3" width="45" customWidth="1"/>
+    <col min="4" max="4" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>161</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>164</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B3" t="s">
-        <v>156</v>
+        <v>166</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>167</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>157</v>
+        <v>168</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -2011,16 +2120,16 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="2" max="2" width="45" customWidth="1"/>
     <col min="3" max="3" width="100" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>17</v>
@@ -2028,57 +2137,57 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>160</v>
-      </c>
-      <c r="B2" t="s">
-        <v>161</v>
+        <v>172</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>173</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>163</v>
-      </c>
-      <c r="B3" t="s">
-        <v>164</v>
+        <v>175</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>176</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>166</v>
-      </c>
-      <c r="B4" t="s">
-        <v>167</v>
+        <v>178</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>179</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>169</v>
-      </c>
-      <c r="B5" t="s">
-        <v>170</v>
+        <v>181</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>182</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>172</v>
-      </c>
-      <c r="B6" t="s">
-        <v>173</v>
+        <v>184</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>185</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -2089,7 +2198,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -2098,90 +2207,106 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>176</v>
+      <c r="A2" s="2" t="s">
+        <v>188</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>178</v>
+      <c r="A3" s="2" t="s">
+        <v>190</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>180</v>
+      <c r="A4" s="2" t="s">
+        <v>192</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>182</v>
+      <c r="A5" s="2" t="s">
+        <v>194</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>184</v>
+      <c r="A6" s="2" t="s">
+        <v>196</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>186</v>
+      <c r="A7" s="2" t="s">
+        <v>198</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>188</v>
+      <c r="A8" s="2" t="s">
+        <v>200</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>190</v>
+      <c r="A9" s="2" t="s">
+        <v>202</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>192</v>
+      <c r="A10" s="2" t="s">
+        <v>204</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>194</v>
+      <c r="A11" s="2" t="s">
+        <v>206</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>195</v>
+        <v>207</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>